<commit_message>
Uluslararası lojistik müşteri aday listesi: TİM 2025 ihracatçıları + ENR 2025 müteahhitleri (Apollo.io zenginleştirmeli)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QANoEyb6T6g5jCfsQADV4W
</commit_message>
<xml_diff>
--- a/musteri-adaylari/lojistik_musteri_aday_listesi.xlsx
+++ b/musteri-adaylari/lojistik_musteri_aday_listesi.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Ihracatci Adaylar" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Ithalatci Adaylar" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Nasil Kullanilir" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Insaat-Taahhut Adaylar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ithalatci Adaylar" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Nasil Kullanilir" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +62,12 @@
       <i val="1"/>
       <color rgb="00C00000"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -112,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -138,6 +145,7 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -529,7 +537,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1906,6 +1913,1535 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>RÖNESANS-BENZERİ ADAYLAR — ULUSLARARASI TÜRK MÜTEAHHİTLERİ (ENR 2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Kaynak: ENR 'Top 250 International Contractors 2025' — Türkiye'den 45 firma (Çin'in 76 firmasının ardından dünya 2.si; 2024'te üstlenilen uluslararası proje değeri 20,8 milyar $ — Ticaret Bakanlığı açıklaması). ENR sırası GERÇEK; Apollo sütunları Apollo.io veritabanından; 'Lojistik açısı' YORUM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Lojistik fırsatı: bu firmalar yurtdışı şantiyelere sürekli ekipman/malzeme sevk eder → proje kargo, ağır/gabari-dışı taşıma, şantiye ikmal zinciri, gümrükleme. Rönesans örneği: Rusya/BDT, Orta Doğu, Avrupa hatları.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Firma</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>ENR 2025 Dünya Sırası</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Apollo: web sitesi</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Apollo: çalışan</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Apollo: merkez</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Lojistik açısı (YORUM)</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Öncelik (YORUM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>ENKA İnşaat</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>enka.com</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>10.000-25.000</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Kazakistan/Irak/Gürcistan santral+altyapı; ağır proje kargo</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Rönesans Holding</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>ronesans.com</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>~32.000</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Ankara</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>REFERANS PROFİL — Rusya/BDT+Orta Doğu şantiye ikmali</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Limak İnşaat</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>limakholding.com</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>~10.000</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Ankara</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Havalimanı/altyapı (Kuveyt, Balkanlar); proje kargo</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Çalık Enerji</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>63</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>calikenerji.com</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>2.000-5.000</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Türkmenistan/Özbekistan enerji santralleri; ağır ekipman</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Esta İnşaat</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>TAV Construction</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Havalimanı inşaatı (Körfez, Afrika); proje kargo</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Ant Yapı</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>88</v>
+      </c>
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr"/>
+      <c r="F12" s="4" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Rusya/BDT+Londra üst yapı; malzeme sevkiyatı</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Gülermak Ağır Sanayi</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>92</v>
+      </c>
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr"/>
+      <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Metro/raylı sistem (Polonya, Hindistan, İngiltere); ağır çelik</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Yapı Merkezi</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>103</v>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>yapimerkezi.com</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>~5.000</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Demiryolu (Tanzanya, Senegal, Suudi Arabistan); ray+vagon+ekipman</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Cengiz İnşaat</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>108</v>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>cengizholding.com.tr</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>~10.000</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Altyapı (Balkanlar, Körfez); ağır makine sevki</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Aslan Yapı</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>109</v>
+      </c>
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Kuzu Grup</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>113</v>
+      </c>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Mapa İnşaat (MNG)</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>115</v>
+      </c>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Afrika/Orta Asya projeleri</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Kolin İnşaat</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>129</v>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>kolin.com.tr</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>5.000-10.000</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Ankara</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Kalyon İnşaat</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>131</v>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>kalyonholding.com</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>~10.000</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Altyapı/enerji (Körfez); proje kargo</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Nurol İnşaat</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>132</v>
+      </c>
+      <c r="D21" s="4" t="inlineStr"/>
+      <c r="E21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>BCM Holding</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>136</v>
+      </c>
+      <c r="D22" s="4" t="inlineStr"/>
+      <c r="E22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>GAP İnşaat (Çalık)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>142</v>
+      </c>
+      <c r="D23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Tekfen İnşaat</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>143</v>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>tekfen.com.tr</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>5.000-10.000</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Petrokimya/boru hattı (Katar, Azerbaycan); ağır çelik konstrüksiyon</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Bayburt Grup</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>145</v>
+      </c>
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Sembol Uluslararası Yatırım</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>146</v>
+      </c>
+      <c r="D26" s="4" t="inlineStr"/>
+      <c r="E26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>İlk İnşaat</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>147</v>
+      </c>
+      <c r="D27" s="4" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Eser İnşaat</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>148</v>
+      </c>
+      <c r="D28" s="4" t="inlineStr"/>
+      <c r="E28" s="4" t="inlineStr"/>
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Metag Grup</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>149</v>
+      </c>
+      <c r="D29" s="4" t="inlineStr"/>
+      <c r="E29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Polat Yol Yapı</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>152</v>
+      </c>
+      <c r="D30" s="4" t="inlineStr"/>
+      <c r="E30" s="4" t="inlineStr"/>
+      <c r="F30" s="4" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Onur Taahhüt (Onur Group)</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>166</v>
+      </c>
+      <c r="D31" s="4" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>Ukrayna/Doğu Avrupa yol-altyapı; makine parkı sevki</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Üstay Yapı</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>171</v>
+      </c>
+      <c r="D32" s="4" t="inlineStr"/>
+      <c r="E32" s="4" t="inlineStr"/>
+      <c r="F32" s="4" t="inlineStr"/>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>IC İçtaş İnşaat</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>173</v>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>ictas.com.tr</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>~5.000</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Rusya (köprü/havalimanı) + altyapı</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>MBD İnşaat</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>174</v>
+      </c>
+      <c r="D34" s="4" t="inlineStr"/>
+      <c r="E34" s="4" t="inlineStr"/>
+      <c r="F34" s="4" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Makyol İnşaat</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>177</v>
+      </c>
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Alarko Taahhüt</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>178</v>
+      </c>
+      <c r="D36" s="4" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Yüksel İnşaat</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>179</v>
+      </c>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>STFA İnşaat</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>185</v>
+      </c>
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="4" t="inlineStr"/>
+      <c r="F38" s="4" t="inlineStr"/>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>Deniz yapıları/liman inşaatı (Körfez); ağır ekipman</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>YDA İnşaat</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>190</v>
+      </c>
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Dekinsan Grup</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>191</v>
+      </c>
+      <c r="D40" s="4" t="inlineStr"/>
+      <c r="E40" s="4" t="inlineStr"/>
+      <c r="F40" s="4" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Summa Turizm Yatırımcılığı</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>192</v>
+      </c>
+      <c r="D41" s="4" t="inlineStr"/>
+      <c r="E41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="inlineStr"/>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>Afrika (Senegal, Kongo...) bina/havalimanı; uzun hat proje kargo</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>İris İnşaat</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>202</v>
+      </c>
+      <c r="D42" s="4" t="inlineStr"/>
+      <c r="E42" s="4" t="inlineStr"/>
+      <c r="F42" s="4" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Tepe İnşaat</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>207</v>
+      </c>
+      <c r="D43" s="4" t="inlineStr"/>
+      <c r="E43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Doğuş İnşaat</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="n">
+        <v>208</v>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>dogusinsaat.com.tr</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>~1.800</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>Metro/altyapı (BDT, Fas)</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Mesa Holding</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="n">
+        <v>210</v>
+      </c>
+      <c r="D45" s="4" t="inlineStr"/>
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Zafer Taahhüt</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="n">
+        <v>212</v>
+      </c>
+      <c r="D46" s="4" t="inlineStr"/>
+      <c r="E46" s="4" t="inlineStr"/>
+      <c r="F46" s="4" t="inlineStr"/>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>SMK Grup</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="n">
+        <v>215</v>
+      </c>
+      <c r="D47" s="4" t="inlineStr"/>
+      <c r="E47" s="4" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr"/>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Dorçe Prefabrik</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="n">
+        <v>229</v>
+      </c>
+      <c r="D48" s="4" t="inlineStr"/>
+      <c r="E48" s="4" t="inlineStr"/>
+      <c r="F48" s="4" t="inlineStr"/>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>Prefabrik modüler yapı İHRACATÇISI — sürekli konteyner/proje yükü</t>
+        </is>
+      </c>
+      <c r="H48" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Özkar İnşaat</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="n">
+        <v>231</v>
+      </c>
+      <c r="D49" s="4" t="inlineStr"/>
+      <c r="E49" s="4" t="inlineStr"/>
+      <c r="F49" s="4" t="inlineStr"/>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>Yurtdışı şantiye ikmali + proje kargo (genel profil)</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Orkun Uluslararası Nakliyat</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="n">
+        <v>234</v>
+      </c>
+      <c r="D50" s="4" t="inlineStr"/>
+      <c r="E50" s="4" t="inlineStr"/>
+      <c r="F50" s="4" t="inlineStr"/>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>⚠ LOJİSTİK FİRMASI — müşteri değil RAKİP; kıyaslama için listede</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="13" t="inlineStr">
+        <is>
+          <t>APOLLO EK BULGULAR (ENR 2025 listesinde yok; Apollo.io veritabanından)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>GAMA Holding</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>gamaholding.com</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>~10.000</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>Ankara</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>Enerji/EPC — santral inşaatı (Orta Doğu, BDT); ağır proje kargo</t>
+        </is>
+      </c>
+      <c r="H53" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Kazancı Holding (Aksa)</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>kazanciholding.com</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>2.000-5.000</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>Enerji/altyapı; jeneratör-santral ekipmanı sevkiyatı (Afrika ağırlıklı)</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Karadeniz Holding (Karpowership)</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>karadenizholding.com</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>~3.000</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>Yüzer santral (Powership) — gemi + ekipman lojistiği, niş proje kargo</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Boş Apollo hücreleri: Apollo koşusunun döndürdüğü 15 firma eşleşmesi dışında kalanlar (VERİ YOK — uydurulmadı). Çalışan sayıları Apollo.io tahminidir.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2267,7 +3803,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Orta ölçek çok-sektör ihracatçı listesi (Apollo 2361 firmalık havuzdan 33 örnek) + filosuz lojistik satış playbook'u
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QANoEyb6T6g5jCfsQADV4W
</commit_message>
<xml_diff>
--- a/musteri-adaylari/lojistik_musteri_aday_listesi.xlsx
+++ b/musteri-adaylari/lojistik_musteri_aday_listesi.xlsx
@@ -9,8 +9,10 @@
   <sheets>
     <sheet name="Ihracatci Adaylar" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Insaat-Taahhut Adaylar" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Ithalatci Adaylar" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Nasil Kullanilir" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Orta Olcek Cok-Sektor" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Ithalatci Adaylar" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Nasil Kullanilir" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Satis Playbook" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -70,7 +72,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -90,6 +92,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E2F3"/>
       </patternFill>
     </fill>
   </fills>
@@ -119,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -146,6 +153,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3447,6 +3456,1089 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ANA AV SAHASI — ORTA ÖLÇEK İHRACATÇILAR (HER SEKTÖR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Kaynak: Apollo.io taraması (09.08.2026) — Türkiye merkezli, 50-1.000 çalışanlı, ihracat yapan üretici havuzu 2.361 firma; aşağıdaki 33'ü Apollo'nun süzdüğü örneklem (çokuluslu şubeleri elendi). Alan adları/çalışan sayıları Apollo tahminidir — arama öncesi siteden teyit et. Filosuz modelde EN VERİMLİ segment budur: lojistik departmanı küçük, spot navlun alıcısı, yeni tedarikçiye açık.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Sektör</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Firma</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Web (Apollo)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Çalışan (Apollo)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Merkez</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Anahtar kelimeler / ihracat pazarı</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>PLASTİK &amp; KAUÇUK/LASTİK</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="n"/>
+      <c r="C5" s="15" t="n"/>
+      <c r="D5" s="15" t="n"/>
+      <c r="E5" s="15" t="n"/>
+      <c r="F5" s="15" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr"/>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Kordsa Teknik Tekstil</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>kordsa.com</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>1.000-2.000</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Lastik güçlendirme; Avrupa+ABD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Polikim Plastik</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>polikim.com.tr</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>100-300</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Gebze</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Enjeksiyon kalıp; Avrupa</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Pimapen (Balplas)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>pimapen.com</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>300-700</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>PVC profil; Avrupa/inşaat</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Gürel Plastik</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>gurelplastik.com.tr</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>50-200</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Bursa</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Teknik plastik, otomotiv parça</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>MAKİNE &amp; EKİPMAN</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Dalgakıran Kompresör</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>dalgakiran.com</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>300-600</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Kompresör; Avrupa + global</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Teksan Jeneratör</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>teksan.com</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>200-500</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Jeneratör; Orta Doğu + Afrika</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr"/>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>FNSS Savunma Sistemleri</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>fnss.com.tr</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>500-1.000</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Ankara</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Zırhlı araç; uluslararası kontratlar</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Nurol Makina</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>nurolvehicles.com</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>200-600</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Ankara</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Savunma araçları; NATO pazarları</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr"/>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>TÜMOSAN Motor ve Traktör</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>tumosan.com.tr</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>400-800</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Konya</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Traktör; ihracat</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr"/>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>REPKON Makina</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>repkon.com</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>100-400</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Metal şekillendirme; savunma+endüstri</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>KİMYA</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="n"/>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="15" t="n"/>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="15" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Organik Kimya</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>organikkimya.com.tr</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>200-500</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Gebze</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Özel kimyasallar/yapıştırıcı; Avrupa</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr"/>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Akkim Kimya</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>akkim.com.tr</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>100-400</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Endüstriyel kimyasallar</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr"/>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Akdeniz Chemson</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>akdenizchemson.com</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>100-300</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Gebze</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>PVC stabilizatör; Avrupa</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr"/>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>İGSAŞ</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>igsas.com.tr</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>300-700</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Gübre; ihracat</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr"/>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>HEKTAŞ</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>hektas.com.tr</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>200-500</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Zirai ilaç; Orta Doğu</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr"/>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Aromsa</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>aromsa.com.tr</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>100-300</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Gebze</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Gıda aroması; Avrupa</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>GIDA İŞLEME</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n"/>
+      <c r="C24" s="15" t="n"/>
+      <c r="D24" s="15" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="15" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr"/>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Kervan Gıda</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>kervan.com.tr</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>300-700</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Şekerleme/jelibon; Avrupa</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr"/>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Ak Gıda</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>akgida.com.tr</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>500-1.000</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Süt ürünleri; FMCG ihracat</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr"/>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Dimes</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>dimes.com.tr</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>300-600</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Tokat</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Meyve suyu; Avrupa</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr"/>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Altıparmak Gıda (Balparmak)</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>altiparmak.com.tr</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>100-300</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Bal/tahin; Orta Doğu+Avrupa</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr"/>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Tadım Gıda</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>tadim.com.tr</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>200-500</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Kuruyemiş; ihracat</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr"/>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Doğadan</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>dogadan.com</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>100-400</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Bitki çayı; Avrupa</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr"/>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Uludağ İçecek</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>uludag.com.tr</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>200-600</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Bursa</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>İçecek; ihracat</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>TEKSTİL</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="n"/>
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="15" t="n"/>
+      <c r="F32" s="15" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr"/>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>ISKO (Sanko Tekstil)</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>iskodenim.com</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>500-1.000</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Gaziantep</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Denim kumaş; global marka</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr"/>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Özdilek Tekstil</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>ozdilek.com.tr</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>300-700</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Bursa</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Ev tekstili; Avrupa</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr"/>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Korteks</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>korteks.com.tr</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>200-600</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Bursa</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Polyester iplik; teknik elyaf</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>MOBİLYA</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="n"/>
+      <c r="C36" s="15" t="n"/>
+      <c r="D36" s="15" t="n"/>
+      <c r="E36" s="15" t="n"/>
+      <c r="F36" s="15" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr"/>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>NURUS Mobilya</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>nurus.com</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>200-500</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Ofis mobilyası; Avrupa/proje</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr"/>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Vivense</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>vivense.com</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>100-300</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Mobilya e-ihracat</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>OTOMOTİV YAN SANAYİ &amp; ARAÇ</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="n"/>
+      <c r="C39" s="15" t="n"/>
+      <c r="D39" s="15" t="n"/>
+      <c r="E39" s="15" t="n"/>
+      <c r="F39" s="15" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr"/>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>TIRSAN Treyler</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>tirsan.com</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>400-800</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Çerkezköy</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Treyler; Avrupa</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr"/>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>BMC</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>bmc.com.tr</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>500-1.000</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>İzmir</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Kamyon/otobüs; Orta Doğu</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr"/>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Bozankaya</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>bozankaya.com</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>200-500</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Ankara</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>Tramvay/elektrikli otobüs; uluslararası</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr"/>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Volta Motor</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>voltamotor.com.tr</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>50-200</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Elektrikli araç/motosiklet</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr"/>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Ege Kimya (kauçuk conta)</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>egekimya.com.tr</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>50-200</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>İzmir</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Otomotiv conta; OEM tedarikçi, Avrupa</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Havuzun tamamı: Apollo'da bu profile uyan 2.361 firma var — bu sayfa örneklemdir. Sonraki turlarda 100'erlik partiler halinde çekilebilir.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3803,7 +4895,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3943,4 +5035,352 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="120" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FİLOSUZ ULUSLARARASI LOJİSTİK — SATIŞ PLAYBOOK (90 GÜN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>KONUMLANDIRMA (filosuz = zayıflık değil, doğru anlatırsan esneklik):</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  "Sabit filo maliyeti taşımıyoruz; 1 tırdan 50 tıra ölçekleniriz, fiyatımız piyasa spotuna yakındır,</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  aracınız bulunamadığında biz buluruz." Güven açığını kapatan üçlü: CMR sigortası + referans dosyası + canlı takip.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>HEDEF SEÇİMİ — kimden iş KOPAR:</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1) Orta ölçek ihracatçı (50-500 çalışan): lojistiği 1-2 kişi yönetir, mevcut nakliyeci aksadığında alternatifi yok → ANA HEDEF</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2) Dış ticaret aracı firmaları: kendi filosu yok, sürekli navlun satın alır → hızlı dönüşüm</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3) Sezonluk yoğunluk (gıda hasat, tekstil sezon, fuar dönemi): taşma (overflow) kapasitesi satılır</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4) İhracata yeni başlayanlar: taşıma + gümrük + evrak danışmanlığı paketi; marj en yüksek</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ✗ Devler (Arçelik, Ford...): yıllık ihale + 60-90 gün vade + fiyat kırdırma → İLK 6 AY GİRME</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>İLK TEMAS (Türkiye gerçeği: telefon &gt; e-posta):</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Arama senaryosu: "X Bey, [firma]dan arıyorum. Almanya'ya haftada kaç araç yüklüyorsunuz?</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Mevcut nakliyecinizden memnunsanız sorun değil — sadece BİR SONRAKİ spot yükünüzde fiyat vermek istiyorum.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tutmazsa bir daha aramam." → Reddedilmesi zor, tek yük iste, sözleşme isteme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  E-posta yalnız arama sonrası teyit + fiyat tablosu olarak gider.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>İŞİ KOPARMA MERDİVENİ:</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. spot yük (marjsız bile al — referans satın alıyorsun) → 3 sorunsuz taşıma → düzenli hat teklifi → aylık mini-sözleşme</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Fiyat değil SORUN çöz: cuma 17:00'de araç bulunamayan yük, gümrükte bekleyen tır, frigo krizi = kapıyı açan an.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>ARAÇ TEDARİĞİ (tırın yok — asıl operasyon burası):</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • 5-10 filo sahibiyle çerçeve anlaşma (UND üyesi taşıyıcılar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Dijital yük borsaları (araç BULMAK için kullan, müşteri bulmak için değil)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Dönüş yükü avcılığı: TR→AB giden aracın dönüşü ucuzdur; iki yönlü eşleştiren kazanır</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Taşıyıcı skorlaması tut (zamanında teslim/hasar/evrak) — senin ürünün taşıma değil GÜVEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>NAKİT GERÇEĞİ (filosuz modelin ölüm riski):</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  İhracatçı 60-90 gün vade ister, taşıyıcı peşine yakın ister → aradaki fark SENİN işletme sermayen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Faktoring/DBS anlaşması olmadan 5+ düzenli müşteriye ÇIKMA. (YORUM — sektör pratiği)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>90 GÜN PLANI:</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  0-30:  3 sektör seç (öneri: plastik + otomotiv yan sanayi + gıda; TR→AB yoğun FTL/parsiyel üretir)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">         100 firmalık liste (bu dosyada hazır) · günde 15 arama · haftada 2 saha ziyareti (Gebze/İkitelli/Bursa OSB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">         5 taşıyıcıyla çerçeve anlaşma</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  30-60: ilk 5 spot yük · WhatsApp konum-takip standardı · referans dosyası (fotoğraf+teslim tutanağı)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  60-90: 3 düzenli müşteri · 1 fuar ziyareti (Plast Eurasia Aralık/İstanbul; ziyaretçi olarak, stand değil)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">         gümrük müşaviri + banka dış ticaret birimiyle karşılıklı yönlendirme ortaklığı</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>KANALLAR (firma bulma):</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • İhracatçı birlikleri üye dizinleri (İKMİB, PAGEV/PAGDER, OAİB, İTKİB) — halka açık</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • OSB firma rehberleri (Gebze, İkitelli, Bursa, Gaziantep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Fuar katılımcı listeleri (katılımcı = kanıtlanmış ihracatçı/ithalatçı)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Apollo.io (bu dosyadaki havuz: 2.361 orta ölçek üretici) + LinkedIn 'dış ticaret müdürü' araması</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Gümrük müşavirleri + nakliye komisyoncusu ağı (komisyon paylaşımlı yönlendirme)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>KPI (gerçekçi huni — YORUM):</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  100 arama → ~20 fiyat teklifi → ~2 yük. Günde 15 arama = ayda ~6 yeni yük denemesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  İlk 90 günde hedef: 3 düzenli müşteri + 10 spot yük. Zengin eden hacim değil TEKRAR ORANI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>ETİKET: Bu sayfa strateji YORUMUDUR (sektör pratiğine dayalı); firma verileri Apollo/TİM/ENR kaynaklı GERÇEKTİR.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>